<commit_message>
all worked with battery and fixed Sleepy's voltage display
</commit_message>
<xml_diff>
--- a/hardware_test/test_results/summary.xlsx
+++ b/hardware_test/test_results/summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,67 +451,77 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>power</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>usb_cam</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>phidgets</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>rplidar</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>realsense</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>arm</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>servo_1</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>servo_2</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>servo_3</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>servo_4</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>servo_5</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>servo_6</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>rplidar_detail</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>fail_detail</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>comment</t>
         </is>
       </c>
     </row>
@@ -591,23 +601,29 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>Total rplidar points: 360, Max measured distance: 4.00 m</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sleepy</t>
+          <t>Lagom</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-06-17T15:51:15</t>
+          <t>2025-06-27T14:31:47</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -627,7 +643,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -672,27 +688,29 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>No rplidar hardware</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t xml:space="preserve">rplidar: ; </t>
-        </is>
-      </c>
+          <t>Total rplidar points: 720, Max measured distance: 5.54 m</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bashful</t>
+          <t>Sleepy</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-06-14T12:27:58</t>
+          <t>2025-06-17T15:51:15</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -717,7 +735,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -757,23 +775,37 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Total rplidar points: 360, Max measured distance: 5.12 m</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>No rplidar hardware</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rplidar: ; </t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Servo5 is loose</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Sneezy</t>
+          <t>Bashful</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2025-06-12T17:22:05</t>
+          <t>2025-06-14T12:27:58</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -838,23 +870,29 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Total rplidar points: 360, Max measured distance: 4.81 m</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Total rplidar points: 360, Max measured distance: 5.12 m</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Vaffor</t>
+          <t>Sneezy</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025-06-25T10:55:19</t>
+          <t>2025-06-12T17:22:05</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -874,7 +912,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -919,27 +957,29 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>No rplidar hardware</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t xml:space="preserve">rplidar: ; </t>
-        </is>
-      </c>
+          <t>Total rplidar points: 360, Max measured distance: 4.81 m</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SnowWhite</t>
+          <t>Vaffor</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025-06-14T11:35:29</t>
+          <t>2025-06-27T15:55:55</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1004,91 +1044,194 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Total rplidar points: 360, Max measured distance: 5.39 m</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr"/>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Total rplidar points: 720, Max measured distance: 6.70 m</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>SnowWhite</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2025-06-14T11:35:29</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Total rplidar points: 360, Max measured distance: 5.39 m</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>No voltage display</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Doc</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" t="n">
         <v>6</v>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>2025-06-13T11:24:15</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>Total rplidar points: 360, Max measured distance: 5.10 m</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>